<commit_message>
Version 1.4.0 Solving the inscription error
</commit_message>
<xml_diff>
--- a/table_temoignages.xlsx
+++ b/table_temoignages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\xlelitebootcamp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA5BBD9-DA02-4CD3-AF93-0EA40476B596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257E8505-AA98-49C3-9C94-6784C7D85F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3975" yWindow="915" windowWidth="21600" windowHeight="13710" xr2:uid="{48DD86A6-B168-4C31-BA06-A0E6F39A0377}"/>
+    <workbookView xWindow="16905" yWindow="0" windowWidth="12000" windowHeight="16305" xr2:uid="{48DD86A6-B168-4C31-BA06-A0E6F39A0377}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Temoignages</t>
   </si>
@@ -46,6 +46,85 @@
   </si>
   <si>
     <t>Fonction</t>
+  </si>
+  <si>
+    <t>Vraiment j'ai été transformé par ce Cabinet Smart Otobos Consulting, la pédagogie de M LEONCE (coach) et le niveau de la formation étaient au summum de nos attentes . Alors vivement la prochaine formation .</t>
+  </si>
+  <si>
+    <t>Auditeur Interne à IBI Groupe</t>
+  </si>
+  <si>
+    <t>Boling Faraba Dembele</t>
+  </si>
+  <si>
+    <t>Bamako, Mali</t>
+  </si>
+  <si>
+    <t>Je recommande vivement #le _cabinet_smart_otobos pour tout besoin de perfectionnement en Excel, Macro et Conception d'outils. Ils ont des formateurs hautement qualifiés dans la formation en Excel basique,avancé ainsi qu'en Macro.
+Merci infiniment à M. LEONCE SODJINOU pour la qualité de la formation qui me permettra de gagner beaucoup plus de temps dans mes tâches quotidiennes.</t>
+  </si>
+  <si>
+    <t>Усман Диабате</t>
+  </si>
+  <si>
+    <t>Mali</t>
+  </si>
+  <si>
+    <t>Merci pour tout, formateur excellent, technique de formation de bonne qualité, contenu riche et varié. De toute les formations en ligne que j'ai déjà faite, la votre est de loin la meilleur et sans comparaison... Thank you so much and I appreciate.</t>
+  </si>
+  <si>
+    <t>Accra</t>
+  </si>
+  <si>
+    <t>Harris Djounga</t>
+  </si>
+  <si>
+    <t>Bonjour tout je remercie le formateur et Son équipe pour la qualité de la formation reçu.
+Toutes mes attentes ont été satisfait à 100%.
+Je recommande fortement la formation à ceux qui n'ont pas encore fait.</t>
+  </si>
+  <si>
+    <t>Abdoulaye Wolomo</t>
+  </si>
+  <si>
+    <t>Grand merci cher formateur, cette formation m'aide beaucoup car je suis en cours de création d'un gestionnaire scolaire.je vous remercie encore</t>
+  </si>
+  <si>
+    <t>Tchiffa Guimbaro Ismael Baare</t>
+  </si>
+  <si>
+    <t>Etudiant</t>
+  </si>
+  <si>
+    <t>Niger</t>
+  </si>
+  <si>
+    <t>Un grand merci au Cabinet Otobos Consulting et particulièrement à notre formateur, Léonce TOUNDE SODJINOU, pour la perfection avec laquelle la formation a été administrée, avec en plus, un coaching participatif et motivateur.
+Je recommande vivement ladite formation tout gestionnaire, responsable administratif et financier, comptable principal, gestionnaire de ressources humaines ... Satisfaction garantie !</t>
+  </si>
+  <si>
+    <t>Abou Ouattara</t>
+  </si>
+  <si>
+    <t>Ouagadougou</t>
+  </si>
+  <si>
+    <t>Bonjour Coach, nous avons été très satisfait de la qualité et temps accorder aux participants. Franchement ça me fait un bout de temps sur les formations en ligne, la votre a été du jamais vu de ma part. Encore merci !</t>
+  </si>
+  <si>
+    <t>Ib Zahara</t>
+  </si>
+  <si>
+    <t>Yopougon, Cote d'ivoire</t>
+  </si>
+  <si>
+    <t>Createur digital</t>
+  </si>
+  <si>
+    <t>Excellente formation avec un formateur très actif et soucieux du détail. Merci a vous et bonne continuation.</t>
+  </si>
+  <si>
+    <t>Yacouba Bengaly</t>
   </si>
 </sst>
 </file>
@@ -81,8 +160,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,26 +479,124 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F96AB795-756C-4647-A75B-C95DB165AC58}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="180" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="195" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 1.5.0 adding real testimonies
</commit_message>
<xml_diff>
--- a/table_temoignages.xlsx
+++ b/table_temoignages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\xlelitebootcamp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257E8505-AA98-49C3-9C94-6784C7D85F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C78980F-EECF-455E-AB04-531634877F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16905" yWindow="0" windowWidth="12000" windowHeight="16305" xr2:uid="{48DD86A6-B168-4C31-BA06-A0E6F39A0377}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{48DD86A6-B168-4C31-BA06-A0E6F39A0377}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -160,16 +160,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -180,6 +205,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4045BF1E-E013-4AB5-A100-15D4BED958C1}" name="Tableau1" displayName="Tableau1" ref="A1:D9" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4">
+  <autoFilter ref="A1:D9" xr:uid="{4045BF1E-E013-4AB5-A100-15D4BED958C1}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{455BC6AE-B61E-4659-8D3D-B81F475BB763}" name="Noms &amp; Prenoms" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{756A4CDF-9D1D-4C46-90BA-6790C413D3D8}" name="Temoignages" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{F37BE90F-821E-4B18-994B-98C1E8B87E22}" name="Pays" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F8CC85E5-8592-4593-83D3-C075CAE7EDAC}" name="Fonction" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -482,17 +520,17 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="18.5703125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="69.5703125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -502,11 +540,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -516,44 +554,44 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="180" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -563,22 +601,22 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="195" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -588,11 +626,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -601,5 +639,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>